<commit_message>
do not use drho or rhosat values from input
</commit_message>
<xml_diff>
--- a/input/input_exp_H2-CO2-T32-P1500.xlsx
+++ b/input/input_exp_H2-CO2-T32-P1500.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/02_UHS EXPERIMENTS/H2 DISPLACEMENT EXPERIMENT/Input/For_github_repo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="716" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9CB0761-CE43-4229-B1E4-63DAAB95191A}"/>
+  <xr:revisionPtr revIDLastSave="723" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0F52014-6E8D-4765-858E-4FAC2F862A1D}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="68">
   <si>
     <t>path</t>
   </si>
@@ -89,9 +89,6 @@
     <t>MMDDYY</t>
   </si>
   <si>
-    <t>kg/m3</t>
-  </si>
-  <si>
     <t>psig</t>
   </si>
   <si>
@@ -107,9 +104,6 @@
     <t>GMT_PGD</t>
   </si>
   <si>
-    <t>vol%</t>
-  </si>
-  <si>
     <t>Key</t>
   </si>
   <si>
@@ -185,27 +179,6 @@
     <t>Q</t>
   </si>
   <si>
-    <t>Experimental data/CF 07-22-25 q1 H2CO2 H SS/</t>
-  </si>
-  <si>
-    <t>Experimental data/CF 07-25-2025 q02 H2CO2 H 32C/</t>
-  </si>
-  <si>
-    <t>Experimental data/CF 07-28-2025 q05 H2CO2 H 32C/</t>
-  </si>
-  <si>
-    <t>rho1sat</t>
-  </si>
-  <si>
-    <t>rho2sat</t>
-  </si>
-  <si>
-    <t>PGD1sat</t>
-  </si>
-  <si>
-    <t>PGD2sat</t>
-  </si>
-  <si>
     <t>GMT-4</t>
   </si>
   <si>
@@ -260,10 +233,13 @@
     <t>long lines before and after core</t>
   </si>
   <si>
-    <t>drho1</t>
-  </si>
-  <si>
-    <t>drho2</t>
+    <t>data/CF-H2-CO2-T32-P1500-H-Q5-R1/</t>
+  </si>
+  <si>
+    <t>data/CF-H2-CO2-T32-P1500-H-Q2-R1/</t>
+  </si>
+  <si>
+    <t>data/CF-H2-CO2-T32-P1500-H-Q1-R1/</t>
   </si>
 </sst>
 </file>
@@ -607,7 +583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI5"/>
+  <dimension ref="A1:AC5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.42578125" customWidth="1"/>
@@ -616,29 +592,28 @@
     <col min="4" max="7" width="7.28515625" customWidth="1"/>
     <col min="8" max="8" width="7.140625" customWidth="1"/>
     <col min="9" max="9" width="7.28515625" customWidth="1"/>
-    <col min="10" max="11" width="7.42578125" customWidth="1"/>
-    <col min="14" max="20" width="10.140625" customWidth="1"/>
-    <col min="21" max="25" width="12.85546875" customWidth="1"/>
-    <col min="26" max="26" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="14.5703125" customWidth="1"/>
-    <col min="29" max="29" width="35.28515625" style="1" customWidth="1"/>
-    <col min="30" max="30" width="21.140625" style="1" customWidth="1"/>
-    <col min="31" max="31" width="21.28515625" style="1" customWidth="1"/>
-    <col min="32" max="32" width="26" style="1" customWidth="1"/>
-    <col min="33" max="33" width="18.28515625" style="2" customWidth="1"/>
-    <col min="34" max="34" width="20.28515625" style="2" customWidth="1"/>
-    <col min="35" max="35" width="11.7109375" customWidth="1"/>
+    <col min="10" max="14" width="10.140625" customWidth="1"/>
+    <col min="15" max="19" width="12.85546875" customWidth="1"/>
+    <col min="20" max="20" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.5703125" customWidth="1"/>
+    <col min="23" max="23" width="35.28515625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="21.140625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="21.28515625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="26" style="1" customWidth="1"/>
+    <col min="27" max="27" width="18.28515625" style="2" customWidth="1"/>
+    <col min="28" max="28" width="20.28515625" style="2" customWidth="1"/>
+    <col min="29" max="29" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D1" t="s">
         <v>13</v>
@@ -650,170 +625,134 @@
         <v>9</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I1" t="s">
         <v>12</v>
       </c>
       <c r="J1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="K1" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="L1" t="s">
         <v>53</v>
       </c>
       <c r="M1" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="N1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="O1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="P1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="Q1" t="s">
+        <v>62</v>
+      </c>
+      <c r="R1" t="s">
+        <v>63</v>
+      </c>
+      <c r="S1" t="s">
         <v>60</v>
       </c>
-      <c r="R1" t="s">
-        <v>62</v>
-      </c>
-      <c r="S1" t="s">
-        <v>63</v>
-      </c>
-      <c r="T1" t="s">
-        <v>65</v>
-      </c>
-      <c r="U1" t="s">
-        <v>67</v>
-      </c>
-      <c r="V1" t="s">
-        <v>70</v>
-      </c>
-      <c r="W1" t="s">
-        <v>71</v>
-      </c>
-      <c r="X1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>69</v>
+      <c r="T1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:35" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="K2" t="s">
-        <v>17</v>
-      </c>
-      <c r="L2" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="M2" t="s">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="N2" t="s">
+        <v>57</v>
+      </c>
+      <c r="P2" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>57</v>
+      </c>
+      <c r="R2" t="s">
+        <v>57</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+    </row>
+    <row r="3" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>23</v>
       </c>
-      <c r="O2" t="s">
-        <v>23</v>
-      </c>
-      <c r="P2" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>61</v>
-      </c>
-      <c r="S2" t="s">
-        <v>64</v>
-      </c>
-      <c r="T2" t="s">
-        <v>66</v>
-      </c>
-      <c r="V2" t="s">
-        <v>66</v>
-      </c>
-      <c r="W2" t="s">
-        <v>66</v>
-      </c>
-      <c r="X2" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="AA2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="AB2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="AG2" s="1"/>
-      <c r="AH2" s="1"/>
-    </row>
-    <row r="3" spans="1:35" ht="75" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>27</v>
-      </c>
       <c r="C3" s="4" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E3" t="s">
         <v>15</v>
@@ -831,96 +770,78 @@
         <v>1</v>
       </c>
       <c r="J3">
-        <v>22.58</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>2.04</v>
+        <v>6</v>
       </c>
       <c r="L3">
-        <v>771.8</v>
+        <v>0.22600000000000001</v>
       </c>
       <c r="M3">
-        <v>5.03</v>
+        <v>202</v>
       </c>
       <c r="N3">
-        <v>100</v>
-      </c>
-      <c r="O3">
-        <v>100</v>
+        <v>57.2</v>
+      </c>
+      <c r="O3" t="s">
+        <v>59</v>
       </c>
       <c r="P3">
-        <v>2</v>
+        <v>60.7</v>
       </c>
       <c r="Q3">
-        <v>6</v>
+        <v>15.9</v>
       </c>
       <c r="R3">
-        <v>0.22600000000000001</v>
-      </c>
-      <c r="S3">
-        <v>202</v>
-      </c>
-      <c r="T3">
-        <v>57.2</v>
-      </c>
-      <c r="U3" t="s">
-        <v>68</v>
+        <v>133.80000000000001</v>
+      </c>
+      <c r="S3" t="s">
+        <v>64</v>
+      </c>
+      <c r="T3" s="3">
+        <v>45860.618796296294</v>
+      </c>
+      <c r="U3" s="3">
+        <v>45860.787499999999</v>
       </c>
       <c r="V3">
-        <v>60.7</v>
-      </c>
-      <c r="W3">
-        <v>15.9</v>
-      </c>
-      <c r="X3">
-        <v>133.80000000000001</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>73</v>
-      </c>
-      <c r="Z3" s="3">
-        <v>45860.618796296294</v>
-      </c>
-      <c r="AA3" s="3">
-        <v>45860.787499999999</v>
-      </c>
-      <c r="AB3">
         <v>1</v>
       </c>
-      <c r="AC3" s="5" t="s">
+      <c r="W3" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC3" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AD3" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="AE3" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="AF3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AG3" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="AI3" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:35" ht="75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
         <v>15</v>
@@ -938,96 +859,78 @@
         <v>1</v>
       </c>
       <c r="J4">
-        <v>22.58</v>
+        <v>2</v>
       </c>
       <c r="K4">
-        <v>2.04</v>
+        <v>6</v>
       </c>
       <c r="L4">
-        <v>771.8</v>
+        <v>0.22600000000000001</v>
       </c>
       <c r="M4">
-        <v>5.03</v>
+        <v>202</v>
       </c>
       <c r="N4">
-        <v>100</v>
-      </c>
-      <c r="O4">
-        <v>100</v>
+        <v>57.2</v>
+      </c>
+      <c r="O4" t="s">
+        <v>59</v>
       </c>
       <c r="P4">
-        <v>2</v>
+        <v>60.7</v>
       </c>
       <c r="Q4">
-        <v>6</v>
+        <v>15.9</v>
       </c>
       <c r="R4">
-        <v>0.22600000000000001</v>
-      </c>
-      <c r="S4">
-        <v>202</v>
-      </c>
-      <c r="T4">
-        <v>57.2</v>
-      </c>
-      <c r="U4" t="s">
-        <v>68</v>
+        <v>133.80000000000001</v>
+      </c>
+      <c r="S4" t="s">
+        <v>64</v>
+      </c>
+      <c r="T4" s="3">
+        <v>45863.485844907409</v>
+      </c>
+      <c r="U4" s="3">
+        <v>45863.578865740739</v>
       </c>
       <c r="V4">
-        <v>60.7</v>
-      </c>
-      <c r="W4">
-        <v>15.9</v>
-      </c>
-      <c r="X4">
-        <v>133.80000000000001</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>73</v>
-      </c>
-      <c r="Z4" s="3">
-        <v>45863.485844907409</v>
-      </c>
-      <c r="AA4" s="3">
-        <v>45863.578865740739</v>
-      </c>
-      <c r="AB4">
         <v>1</v>
       </c>
-      <c r="AC4" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD4" s="5" t="s">
+      <c r="W4" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="AE4" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="AF4" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="AG4" s="6" t="s">
+      <c r="AC4" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AH4" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="AI4" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5" spans="1:35" ht="75" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="C5" s="4" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
         <v>15</v>
@@ -1045,82 +948,64 @@
         <v>1</v>
       </c>
       <c r="J5">
-        <v>22.58</v>
+        <v>2</v>
       </c>
       <c r="K5">
-        <v>2.04</v>
+        <v>6</v>
       </c>
       <c r="L5">
-        <v>771.8</v>
+        <v>0.22600000000000001</v>
       </c>
       <c r="M5">
-        <v>5.03</v>
+        <v>202</v>
       </c>
       <c r="N5">
-        <v>100</v>
-      </c>
-      <c r="O5">
-        <v>100</v>
+        <v>57.2</v>
+      </c>
+      <c r="O5" t="s">
+        <v>59</v>
       </c>
       <c r="P5">
-        <v>2</v>
+        <v>60.7</v>
       </c>
       <c r="Q5">
-        <v>6</v>
+        <v>15.9</v>
       </c>
       <c r="R5">
-        <v>0.22600000000000001</v>
-      </c>
-      <c r="S5">
-        <v>202</v>
-      </c>
-      <c r="T5">
-        <v>57.2</v>
-      </c>
-      <c r="U5" t="s">
-        <v>68</v>
+        <v>133.80000000000001</v>
+      </c>
+      <c r="S5" t="s">
+        <v>64</v>
+      </c>
+      <c r="T5" s="3">
+        <v>45866.503113425926</v>
+      </c>
+      <c r="U5" s="3">
+        <v>45866.552349537036</v>
       </c>
       <c r="V5">
-        <v>60.7</v>
-      </c>
-      <c r="W5">
-        <v>15.9</v>
-      </c>
-      <c r="X5">
-        <v>133.80000000000001</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>73</v>
-      </c>
-      <c r="Z5" s="3">
-        <v>45866.503113425926</v>
-      </c>
-      <c r="AA5" s="3">
-        <v>45866.552349537036</v>
-      </c>
-      <c r="AB5">
         <v>1</v>
       </c>
-      <c r="AC5" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD5" s="1" t="s">
+      <c r="W5" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="X5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AE5" s="1" t="s">
+      <c r="AB5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AF5" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AG5" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="AH5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="AI5" s="1" t="s">
-        <v>56</v>
+      <c r="AC5" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed Vlines after and before to corrected values
</commit_message>
<xml_diff>
--- a/input/input_exp_H2-CO2-T32-P1500.xlsx
+++ b/input/input_exp_H2-CO2-T32-P1500.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="723" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0F52014-6E8D-4765-858E-4FAC2F862A1D}"/>
+  <xr:revisionPtr revIDLastSave="735" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E15EF4D-C0D0-4DD0-8E70-65F8981862FF}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -593,7 +593,8 @@
     <col min="8" max="8" width="7.140625" customWidth="1"/>
     <col min="9" max="9" width="7.28515625" customWidth="1"/>
     <col min="10" max="14" width="10.140625" customWidth="1"/>
-    <col min="15" max="19" width="12.85546875" customWidth="1"/>
+    <col min="15" max="18" width="12.85546875" customWidth="1"/>
+    <col min="19" max="19" width="30.28515625" customWidth="1"/>
     <col min="20" max="20" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="14.5703125" customWidth="1"/>
     <col min="23" max="23" width="35.28515625" style="1" customWidth="1"/>
@@ -788,7 +789,7 @@
         <v>59</v>
       </c>
       <c r="P3">
-        <v>60.7</v>
+        <v>30.8</v>
       </c>
       <c r="Q3">
         <v>15.9</v>
@@ -877,7 +878,7 @@
         <v>59</v>
       </c>
       <c r="P4">
-        <v>60.7</v>
+        <v>30.8</v>
       </c>
       <c r="Q4">
         <v>15.9</v>
@@ -966,7 +967,7 @@
         <v>59</v>
       </c>
       <c r="P5">
-        <v>60.7</v>
+        <v>30.8</v>
       </c>
       <c r="Q5">
         <v>15.9</v>

</xml_diff>

<commit_message>
main Data Extract with changes in input and import after import function was changed during main Cal modifications
</commit_message>
<xml_diff>
--- a/input/input_exp_H2-CO2-T32-P1500.xlsx
+++ b/input/input_exp_H2-CO2-T32-P1500.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="739" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{991C1363-AD9D-407E-B0A9-4F5E3EAB6344}"/>
+  <xr:revisionPtr revIDLastSave="754" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B14F77E6-40A7-4028-80E3-482BF8C89AD7}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="71">
   <si>
     <t>path</t>
   </si>
@@ -240,6 +240,15 @@
   </si>
   <si>
     <t>data/CF-H2-CO2-T32-P1500-H-Q1-R1/</t>
+  </si>
+  <si>
+    <t>workingPump</t>
+  </si>
+  <si>
+    <t>cushionPump</t>
+  </si>
+  <si>
+    <t>confiningPump</t>
   </si>
 </sst>
 </file>
@@ -583,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC5"/>
+  <dimension ref="A1:AF5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.42578125" customWidth="1"/>
@@ -594,19 +603,19 @@
     <col min="9" max="9" width="7.28515625" customWidth="1"/>
     <col min="10" max="14" width="10.140625" customWidth="1"/>
     <col min="15" max="18" width="12.85546875" customWidth="1"/>
-    <col min="19" max="19" width="30.28515625" customWidth="1"/>
-    <col min="20" max="20" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.5703125" customWidth="1"/>
-    <col min="23" max="23" width="35.28515625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="21.140625" style="1" customWidth="1"/>
-    <col min="25" max="25" width="21.28515625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="26" style="1" customWidth="1"/>
-    <col min="27" max="27" width="18.28515625" style="2" customWidth="1"/>
-    <col min="28" max="28" width="20.28515625" style="2" customWidth="1"/>
-    <col min="29" max="29" width="11.7109375" customWidth="1"/>
+    <col min="19" max="22" width="30.28515625" customWidth="1"/>
+    <col min="23" max="23" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14.5703125" customWidth="1"/>
+    <col min="26" max="26" width="35.28515625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="21.140625" style="1" customWidth="1"/>
+    <col min="28" max="28" width="21.28515625" style="1" customWidth="1"/>
+    <col min="29" max="29" width="26" style="1" customWidth="1"/>
+    <col min="30" max="30" width="18.28515625" style="2" customWidth="1"/>
+    <col min="31" max="31" width="20.28515625" style="2" customWidth="1"/>
+    <col min="32" max="32" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -664,38 +673,47 @@
       <c r="S1" t="s">
         <v>60</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
+        <v>68</v>
+      </c>
+      <c r="U1" t="s">
+        <v>69</v>
+      </c>
+      <c r="V1" t="s">
+        <v>70</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:29" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>16</v>
       </c>
@@ -730,19 +748,19 @@
       <c r="R2" t="s">
         <v>57</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="X2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="AA2" s="1"/>
-      <c r="AB2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="1"/>
     </row>
-    <row r="3" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -800,38 +818,47 @@
       <c r="S3" t="s">
         <v>64</v>
       </c>
-      <c r="T3" s="3">
+      <c r="T3">
+        <v>1</v>
+      </c>
+      <c r="U3">
+        <v>2</v>
+      </c>
+      <c r="V3">
+        <v>3</v>
+      </c>
+      <c r="W3" s="3">
         <v>45860.618796296294</v>
       </c>
-      <c r="U3" s="3">
+      <c r="X3" s="3">
         <v>45860.787499999999</v>
       </c>
-      <c r="V3">
+      <c r="Y3">
         <v>1</v>
       </c>
-      <c r="W3" s="5" t="s">
+      <c r="Z3" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="X3" s="5" t="s">
+      <c r="AA3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y3" s="5" t="s">
+      <c r="AB3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="Z3" s="5" t="s">
+      <c r="AC3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="AA3" s="6" t="s">
+      <c r="AD3" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="AB3" s="6" t="s">
+      <c r="AE3" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="AC3" s="1" t="s">
+      <c r="AF3" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -889,38 +916,47 @@
       <c r="S4" t="s">
         <v>64</v>
       </c>
-      <c r="T4" s="3">
+      <c r="T4">
+        <v>1</v>
+      </c>
+      <c r="U4">
+        <v>2</v>
+      </c>
+      <c r="V4">
+        <v>3</v>
+      </c>
+      <c r="W4" s="3">
         <v>45863.485844907409</v>
       </c>
-      <c r="U4" s="3">
+      <c r="X4" s="3">
         <v>45863.578865740739</v>
       </c>
-      <c r="V4">
+      <c r="Y4">
         <v>1</v>
       </c>
-      <c r="W4" s="5" t="s">
+      <c r="Z4" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="X4" s="5" t="s">
+      <c r="AA4" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="Y4" s="5" t="s">
+      <c r="AB4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="Z4" s="5" t="s">
+      <c r="AC4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AA4" s="6" t="s">
+      <c r="AD4" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="AB4" s="6" t="s">
+      <c r="AE4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="AC4" s="1" t="s">
+      <c r="AF4" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:29" ht="75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:32" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -978,34 +1014,43 @@
       <c r="S5" t="s">
         <v>64</v>
       </c>
-      <c r="T5" s="3">
+      <c r="T5">
+        <v>1</v>
+      </c>
+      <c r="U5">
+        <v>2</v>
+      </c>
+      <c r="V5">
+        <v>3</v>
+      </c>
+      <c r="W5" s="3">
         <v>45866.503113425926</v>
       </c>
-      <c r="U5" s="3">
+      <c r="X5" s="3">
         <v>45866.552349537036</v>
       </c>
-      <c r="V5">
+      <c r="Y5">
         <v>1</v>
       </c>
-      <c r="W5" s="5" t="s">
+      <c r="Z5" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="X5" s="1" t="s">
+      <c r="AA5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="Y5" s="1" t="s">
+      <c r="AB5" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="Z5" s="1" t="s">
+      <c r="AC5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AA5" s="2" t="s">
+      <c r="AD5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AB5" s="2" t="s">
+      <c r="AE5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AC5" s="1" t="s">
+      <c r="AF5" s="1" t="s">
         <v>47</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add and update input files
</commit_message>
<xml_diff>
--- a/input/input_exp_H2-CO2-T32-P1500.xlsx
+++ b/input/input_exp_H2-CO2-T32-P1500.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="754" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B14F77E6-40A7-4028-80E3-482BF8C89AD7}"/>
+  <xr:revisionPtr revIDLastSave="770" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0AB5C2A7-01E6-4CE8-AB4E-3EC7722A9DFB}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
   <si>
     <t>path</t>
   </si>
@@ -249,6 +249,15 @@
   </si>
   <si>
     <t>confiningPump</t>
+  </si>
+  <si>
+    <t>% mol</t>
+  </si>
+  <si>
+    <t>C1init</t>
+  </si>
+  <si>
+    <t>C1j</t>
   </si>
 </sst>
 </file>
@@ -592,30 +601,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AF5"/>
+  <dimension ref="A1:AH5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.42578125" customWidth="1"/>
     <col min="2" max="2" width="9.85546875" style="4" customWidth="1"/>
     <col min="3" max="3" width="7.7109375" style="4" customWidth="1"/>
     <col min="4" max="7" width="7.28515625" customWidth="1"/>
-    <col min="8" max="8" width="7.140625" customWidth="1"/>
-    <col min="9" max="9" width="7.28515625" customWidth="1"/>
-    <col min="10" max="14" width="10.140625" customWidth="1"/>
-    <col min="15" max="18" width="12.85546875" customWidth="1"/>
-    <col min="19" max="22" width="30.28515625" customWidth="1"/>
-    <col min="23" max="23" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="14.5703125" customWidth="1"/>
-    <col min="26" max="26" width="35.28515625" style="1" customWidth="1"/>
-    <col min="27" max="27" width="21.140625" style="1" customWidth="1"/>
-    <col min="28" max="28" width="21.28515625" style="1" customWidth="1"/>
-    <col min="29" max="29" width="26" style="1" customWidth="1"/>
-    <col min="30" max="30" width="18.28515625" style="2" customWidth="1"/>
-    <col min="31" max="31" width="20.28515625" style="2" customWidth="1"/>
-    <col min="32" max="32" width="11.7109375" customWidth="1"/>
+    <col min="8" max="10" width="7.140625" customWidth="1"/>
+    <col min="11" max="11" width="7.28515625" customWidth="1"/>
+    <col min="12" max="16" width="10.140625" customWidth="1"/>
+    <col min="17" max="20" width="12.85546875" customWidth="1"/>
+    <col min="21" max="24" width="30.28515625" customWidth="1"/>
+    <col min="25" max="25" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.5703125" customWidth="1"/>
+    <col min="28" max="28" width="35.28515625" style="1" customWidth="1"/>
+    <col min="29" max="29" width="21.140625" style="1" customWidth="1"/>
+    <col min="30" max="30" width="21.28515625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="26" style="1" customWidth="1"/>
+    <col min="32" max="32" width="18.28515625" style="2" customWidth="1"/>
+    <col min="33" max="33" width="20.28515625" style="2" customWidth="1"/>
+    <col min="34" max="34" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -640,80 +649,86 @@
       <c r="H1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K1" t="s">
         <v>12</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>50</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>51</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>53</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>54</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>56</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>58</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>61</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="S1" t="s">
         <v>62</v>
       </c>
-      <c r="R1" t="s">
+      <c r="T1" t="s">
         <v>63</v>
       </c>
-      <c r="S1" t="s">
+      <c r="U1" t="s">
         <v>60</v>
       </c>
-      <c r="T1" t="s">
+      <c r="V1" t="s">
         <v>68</v>
       </c>
-      <c r="U1" t="s">
+      <c r="W1" t="s">
         <v>69</v>
       </c>
-      <c r="V1" t="s">
+      <c r="X1" t="s">
         <v>70</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:32" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:34" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>16</v>
       </c>
@@ -726,41 +741,47 @@
       <c r="H2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="1"/>
-      <c r="J2" t="s">
+      <c r="I2" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="K2" s="1"/>
+      <c r="L2" t="s">
         <v>52</v>
       </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
         <v>52</v>
       </c>
-      <c r="M2" t="s">
+      <c r="O2" t="s">
         <v>55</v>
-      </c>
-      <c r="N2" t="s">
-        <v>57</v>
       </c>
       <c r="P2" t="s">
         <v>57</v>
       </c>
-      <c r="Q2" t="s">
-        <v>57</v>
-      </c>
       <c r="R2" t="s">
         <v>57</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="S2" t="s">
+        <v>57</v>
+      </c>
+      <c r="T2" t="s">
+        <v>57</v>
+      </c>
+      <c r="Y2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="Z2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="Y2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="AD2" s="1"/>
-      <c r="AE2" s="1"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
     </row>
-    <row r="3" spans="1:32" ht="75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:34" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -786,79 +807,85 @@
         <v>1</v>
       </c>
       <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>100</v>
+      </c>
+      <c r="K3">
         <v>1</v>
       </c>
-      <c r="J3">
+      <c r="L3">
         <v>2</v>
       </c>
-      <c r="K3">
+      <c r="M3">
         <v>6</v>
       </c>
-      <c r="L3">
+      <c r="N3">
         <v>0.193</v>
       </c>
-      <c r="M3">
+      <c r="O3">
         <v>202</v>
       </c>
-      <c r="N3">
+      <c r="P3">
         <v>59.8</v>
       </c>
-      <c r="O3" t="s">
+      <c r="Q3" t="s">
         <v>59</v>
       </c>
-      <c r="P3">
+      <c r="R3">
         <v>30.8</v>
       </c>
-      <c r="Q3">
+      <c r="S3">
         <v>15.9</v>
       </c>
-      <c r="R3">
+      <c r="T3">
         <v>133.80000000000001</v>
       </c>
-      <c r="S3" t="s">
+      <c r="U3" t="s">
         <v>64</v>
       </c>
-      <c r="T3">
+      <c r="V3">
         <v>1</v>
       </c>
-      <c r="U3">
+      <c r="W3">
         <v>2</v>
       </c>
-      <c r="V3">
+      <c r="X3">
         <v>3</v>
       </c>
-      <c r="W3" s="3">
+      <c r="Y3" s="3">
         <v>45860.618796296294</v>
       </c>
-      <c r="X3" s="3">
+      <c r="Z3" s="3">
         <v>45860.787499999999</v>
       </c>
-      <c r="Y3">
+      <c r="AA3">
         <v>1</v>
       </c>
-      <c r="Z3" s="5" t="s">
+      <c r="AB3" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="AA3" s="5" t="s">
+      <c r="AC3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AB3" s="5" t="s">
+      <c r="AD3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AC3" s="5" t="s">
+      <c r="AE3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="AD3" s="6" t="s">
+      <c r="AF3" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="AE3" s="6" t="s">
+      <c r="AG3" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="AF3" s="1" t="s">
+      <c r="AH3" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:32" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:34" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -884,79 +911,85 @@
         <v>2</v>
       </c>
       <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>100</v>
+      </c>
+      <c r="K4">
         <v>1</v>
       </c>
-      <c r="J4">
+      <c r="L4">
         <v>2</v>
       </c>
-      <c r="K4">
+      <c r="M4">
         <v>6</v>
       </c>
-      <c r="L4">
+      <c r="N4">
         <v>0.193</v>
       </c>
-      <c r="M4">
+      <c r="O4">
         <v>202</v>
       </c>
-      <c r="N4">
+      <c r="P4">
         <v>59.8</v>
       </c>
-      <c r="O4" t="s">
+      <c r="Q4" t="s">
         <v>59</v>
       </c>
-      <c r="P4">
+      <c r="R4">
         <v>30.8</v>
       </c>
-      <c r="Q4">
+      <c r="S4">
         <v>15.9</v>
       </c>
-      <c r="R4">
+      <c r="T4">
         <v>133.80000000000001</v>
       </c>
-      <c r="S4" t="s">
+      <c r="U4" t="s">
         <v>64</v>
       </c>
-      <c r="T4">
+      <c r="V4">
         <v>1</v>
       </c>
-      <c r="U4">
+      <c r="W4">
         <v>2</v>
       </c>
-      <c r="V4">
+      <c r="X4">
         <v>3</v>
       </c>
-      <c r="W4" s="3">
+      <c r="Y4" s="3">
         <v>45863.485844907409</v>
       </c>
-      <c r="X4" s="3">
+      <c r="Z4" s="3">
         <v>45863.578865740739</v>
       </c>
-      <c r="Y4">
+      <c r="AA4">
         <v>1</v>
       </c>
-      <c r="Z4" s="5" t="s">
+      <c r="AB4" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="AA4" s="5" t="s">
+      <c r="AC4" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="AB4" s="5" t="s">
+      <c r="AD4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AC4" s="5" t="s">
+      <c r="AE4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AD4" s="6" t="s">
+      <c r="AF4" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="AE4" s="6" t="s">
+      <c r="AG4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="AF4" s="1" t="s">
+      <c r="AH4" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:32" ht="75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:34" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -982,75 +1015,81 @@
         <v>5</v>
       </c>
       <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>100</v>
+      </c>
+      <c r="K5">
         <v>1</v>
       </c>
-      <c r="J5">
+      <c r="L5">
         <v>2</v>
       </c>
-      <c r="K5">
+      <c r="M5">
         <v>6</v>
       </c>
-      <c r="L5">
+      <c r="N5">
         <v>0.193</v>
       </c>
-      <c r="M5">
+      <c r="O5">
         <v>202</v>
       </c>
-      <c r="N5">
+      <c r="P5">
         <v>59.8</v>
       </c>
-      <c r="O5" t="s">
+      <c r="Q5" t="s">
         <v>59</v>
       </c>
-      <c r="P5">
+      <c r="R5">
         <v>30.8</v>
       </c>
-      <c r="Q5">
+      <c r="S5">
         <v>15.9</v>
       </c>
-      <c r="R5">
+      <c r="T5">
         <v>133.80000000000001</v>
       </c>
-      <c r="S5" t="s">
+      <c r="U5" t="s">
         <v>64</v>
       </c>
-      <c r="T5">
+      <c r="V5">
         <v>1</v>
       </c>
-      <c r="U5">
+      <c r="W5">
         <v>2</v>
       </c>
-      <c r="V5">
+      <c r="X5">
         <v>3</v>
       </c>
-      <c r="W5" s="3">
+      <c r="Y5" s="3">
         <v>45866.503113425926</v>
       </c>
-      <c r="X5" s="3">
+      <c r="Z5" s="3">
         <v>45866.552349537036</v>
       </c>
-      <c r="Y5">
+      <c r="AA5">
         <v>1</v>
       </c>
-      <c r="Z5" s="5" t="s">
+      <c r="AB5" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="AA5" s="1" t="s">
+      <c r="AC5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AB5" s="1" t="s">
+      <c r="AD5" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AC5" s="1" t="s">
+      <c r="AE5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AD5" s="2" t="s">
+      <c r="AF5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AE5" s="2" t="s">
+      <c r="AG5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AF5" s="1" t="s">
+      <c r="AH5" s="1" t="s">
         <v>47</v>
       </c>
     </row>

</xml_diff>

<commit_message>
area and lines diameter added
</commit_message>
<xml_diff>
--- a/input/input_exp_H2-CO2-T32-P1500.xlsx
+++ b/input/input_exp_H2-CO2-T32-P1500.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="770" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0AB5C2A7-01E6-4CE8-AB4E-3EC7722A9DFB}"/>
+  <xr:revisionPtr revIDLastSave="778" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{592E19CB-7FCC-4F7A-9B2A-5A05225908B0}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="76">
   <si>
     <t>path</t>
   </si>
@@ -258,6 +258,12 @@
   </si>
   <si>
     <t>C1j</t>
+  </si>
+  <si>
+    <t>cm</t>
+  </si>
+  <si>
+    <t>IDlines</t>
   </si>
 </sst>
 </file>
@@ -601,30 +607,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AI5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="7.7109375" style="4" customWidth="1"/>
-    <col min="4" max="7" width="7.28515625" customWidth="1"/>
-    <col min="8" max="10" width="7.140625" customWidth="1"/>
-    <col min="11" max="11" width="7.28515625" customWidth="1"/>
-    <col min="12" max="16" width="10.140625" customWidth="1"/>
-    <col min="17" max="20" width="12.85546875" customWidth="1"/>
-    <col min="21" max="24" width="30.28515625" customWidth="1"/>
-    <col min="25" max="25" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.5703125" customWidth="1"/>
-    <col min="28" max="28" width="35.28515625" style="1" customWidth="1"/>
-    <col min="29" max="29" width="21.140625" style="1" customWidth="1"/>
-    <col min="30" max="30" width="21.28515625" style="1" customWidth="1"/>
-    <col min="31" max="31" width="26" style="1" customWidth="1"/>
-    <col min="32" max="32" width="18.28515625" style="2" customWidth="1"/>
-    <col min="33" max="33" width="20.28515625" style="2" customWidth="1"/>
-    <col min="34" max="34" width="11.7109375" customWidth="1"/>
+    <col min="1" max="1" width="30.44140625" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="7.6640625" style="4" customWidth="1"/>
+    <col min="4" max="7" width="7.33203125" customWidth="1"/>
+    <col min="8" max="10" width="7.109375" customWidth="1"/>
+    <col min="11" max="11" width="7.33203125" customWidth="1"/>
+    <col min="12" max="16" width="10.109375" customWidth="1"/>
+    <col min="17" max="21" width="12.88671875" customWidth="1"/>
+    <col min="22" max="25" width="30.33203125" customWidth="1"/>
+    <col min="26" max="26" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.5546875" customWidth="1"/>
+    <col min="29" max="29" width="35.33203125" style="1" customWidth="1"/>
+    <col min="30" max="30" width="21.109375" style="1" customWidth="1"/>
+    <col min="31" max="31" width="21.33203125" style="1" customWidth="1"/>
+    <col min="32" max="32" width="26" style="1" customWidth="1"/>
+    <col min="33" max="33" width="18.33203125" style="2" customWidth="1"/>
+    <col min="34" max="34" width="20.33203125" style="2" customWidth="1"/>
+    <col min="35" max="35" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -677,58 +683,61 @@
         <v>58</v>
       </c>
       <c r="R1" t="s">
+        <v>75</v>
+      </c>
+      <c r="S1" t="s">
         <v>61</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>62</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>63</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>60</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>68</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>69</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>70</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
         <v>16</v>
       </c>
@@ -761,7 +770,7 @@
         <v>57</v>
       </c>
       <c r="R2" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="S2" t="s">
         <v>57</v>
@@ -769,19 +778,22 @@
       <c r="T2" t="s">
         <v>57</v>
       </c>
-      <c r="Y2" s="1" t="s">
-        <v>19</v>
+      <c r="U2" t="s">
+        <v>57</v>
       </c>
       <c r="Z2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="AA2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="AF2" s="1"/>
       <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
     </row>
-    <row r="3" spans="1:34" ht="75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -834,58 +846,61 @@
         <v>59</v>
       </c>
       <c r="R3">
+        <v>0.29599999999999999</v>
+      </c>
+      <c r="S3">
         <v>30.8</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <v>15.9</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>133.80000000000001</v>
       </c>
-      <c r="U3" t="s">
+      <c r="V3" t="s">
         <v>64</v>
       </c>
-      <c r="V3">
+      <c r="W3">
         <v>1</v>
       </c>
-      <c r="W3">
+      <c r="X3">
         <v>2</v>
       </c>
-      <c r="X3">
+      <c r="Y3">
         <v>3</v>
       </c>
-      <c r="Y3" s="3">
+      <c r="Z3" s="3">
         <v>45860.618796296294</v>
       </c>
-      <c r="Z3" s="3">
+      <c r="AA3" s="3">
         <v>45860.787499999999</v>
       </c>
-      <c r="AA3">
+      <c r="AB3">
         <v>1</v>
       </c>
-      <c r="AB3" s="5" t="s">
+      <c r="AC3" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="AC3" s="5" t="s">
+      <c r="AD3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AD3" s="5" t="s">
+      <c r="AE3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AE3" s="5" t="s">
+      <c r="AF3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="AF3" s="6" t="s">
+      <c r="AG3" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="AG3" s="6" t="s">
+      <c r="AH3" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="AH3" s="1" t="s">
+      <c r="AI3" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:34" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -938,58 +953,61 @@
         <v>59</v>
       </c>
       <c r="R4">
+        <v>0.29599999999999999</v>
+      </c>
+      <c r="S4">
         <v>30.8</v>
       </c>
-      <c r="S4">
+      <c r="T4">
         <v>15.9</v>
       </c>
-      <c r="T4">
+      <c r="U4">
         <v>133.80000000000001</v>
       </c>
-      <c r="U4" t="s">
+      <c r="V4" t="s">
         <v>64</v>
       </c>
-      <c r="V4">
+      <c r="W4">
         <v>1</v>
       </c>
-      <c r="W4">
+      <c r="X4">
         <v>2</v>
       </c>
-      <c r="X4">
+      <c r="Y4">
         <v>3</v>
       </c>
-      <c r="Y4" s="3">
+      <c r="Z4" s="3">
         <v>45863.485844907409</v>
       </c>
-      <c r="Z4" s="3">
+      <c r="AA4" s="3">
         <v>45863.578865740739</v>
       </c>
-      <c r="AA4">
+      <c r="AB4">
         <v>1</v>
       </c>
-      <c r="AB4" s="5" t="s">
+      <c r="AC4" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="AC4" s="5" t="s">
+      <c r="AD4" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="AD4" s="5" t="s">
+      <c r="AE4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AE4" s="5" t="s">
+      <c r="AF4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AF4" s="6" t="s">
+      <c r="AG4" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="AG4" s="6" t="s">
+      <c r="AH4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="AH4" s="1" t="s">
+      <c r="AI4" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:34" ht="75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" ht="72" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -1042,54 +1060,57 @@
         <v>59</v>
       </c>
       <c r="R5">
+        <v>0.29599999999999999</v>
+      </c>
+      <c r="S5">
         <v>30.8</v>
       </c>
-      <c r="S5">
+      <c r="T5">
         <v>15.9</v>
       </c>
-      <c r="T5">
+      <c r="U5">
         <v>133.80000000000001</v>
       </c>
-      <c r="U5" t="s">
+      <c r="V5" t="s">
         <v>64</v>
       </c>
-      <c r="V5">
+      <c r="W5">
         <v>1</v>
       </c>
-      <c r="W5">
+      <c r="X5">
         <v>2</v>
       </c>
-      <c r="X5">
+      <c r="Y5">
         <v>3</v>
       </c>
-      <c r="Y5" s="3">
+      <c r="Z5" s="3">
         <v>45866.503113425926</v>
       </c>
-      <c r="Z5" s="3">
+      <c r="AA5" s="3">
         <v>45866.552349537036</v>
       </c>
-      <c r="AA5">
+      <c r="AB5">
         <v>1</v>
       </c>
-      <c r="AB5" s="5" t="s">
+      <c r="AC5" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="AC5" s="1" t="s">
+      <c r="AD5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AD5" s="1" t="s">
+      <c r="AE5" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AE5" s="1" t="s">
+      <c r="AF5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AF5" s="2" t="s">
+      <c r="AG5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AG5" s="2" t="s">
+      <c r="AH5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AH5" s="1" t="s">
+      <c r="AI5" s="1" t="s">
         <v>47</v>
       </c>
     </row>

</xml_diff>

<commit_message>
cahnges after main Data Extract with input exps changed in Vbefore and affter
</commit_message>
<xml_diff>
--- a/input/input_exp_H2-CO2-T32-P1500.xlsx
+++ b/input/input_exp_H2-CO2-T32-P1500.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="778" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{592E19CB-7FCC-4F7A-9B2A-5A05225908B0}"/>
+  <xr:revisionPtr revIDLastSave="791" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12C60C97-F58A-42E1-A10C-49BBDCC69CDA}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -608,29 +608,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AI5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="7.6640625" style="4" customWidth="1"/>
-    <col min="4" max="7" width="7.33203125" customWidth="1"/>
-    <col min="8" max="10" width="7.109375" customWidth="1"/>
-    <col min="11" max="11" width="7.33203125" customWidth="1"/>
-    <col min="12" max="16" width="10.109375" customWidth="1"/>
-    <col min="17" max="21" width="12.88671875" customWidth="1"/>
-    <col min="22" max="25" width="30.33203125" customWidth="1"/>
-    <col min="26" max="26" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="14.5546875" customWidth="1"/>
-    <col min="29" max="29" width="35.33203125" style="1" customWidth="1"/>
-    <col min="30" max="30" width="21.109375" style="1" customWidth="1"/>
-    <col min="31" max="31" width="21.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="30.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="7.7109375" style="4" customWidth="1"/>
+    <col min="4" max="7" width="7.28515625" customWidth="1"/>
+    <col min="8" max="10" width="7.140625" customWidth="1"/>
+    <col min="11" max="11" width="7.28515625" customWidth="1"/>
+    <col min="12" max="16" width="10.140625" customWidth="1"/>
+    <col min="17" max="21" width="12.85546875" customWidth="1"/>
+    <col min="22" max="25" width="30.28515625" customWidth="1"/>
+    <col min="26" max="26" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.5703125" customWidth="1"/>
+    <col min="29" max="29" width="35.28515625" style="1" customWidth="1"/>
+    <col min="30" max="30" width="21.140625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="21.28515625" style="1" customWidth="1"/>
     <col min="32" max="32" width="26" style="1" customWidth="1"/>
-    <col min="33" max="33" width="18.33203125" style="2" customWidth="1"/>
-    <col min="34" max="34" width="20.33203125" style="2" customWidth="1"/>
-    <col min="35" max="35" width="11.6640625" customWidth="1"/>
+    <col min="33" max="33" width="18.28515625" style="2" customWidth="1"/>
+    <col min="34" max="34" width="20.28515625" style="2" customWidth="1"/>
+    <col min="35" max="35" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -737,7 +737,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:35" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:35" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>16</v>
       </c>
@@ -793,7 +793,7 @@
       <c r="AG2" s="1"/>
       <c r="AH2" s="1"/>
     </row>
-    <row r="3" spans="1:35" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:35" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -846,16 +846,16 @@
         <v>59</v>
       </c>
       <c r="R3">
-        <v>0.29599999999999999</v>
+        <v>0.29399999999999998</v>
       </c>
       <c r="S3">
-        <v>30.8</v>
+        <v>30.9</v>
       </c>
       <c r="T3">
-        <v>15.9</v>
+        <v>13.1</v>
       </c>
       <c r="U3">
-        <v>133.80000000000001</v>
+        <v>103.8</v>
       </c>
       <c r="V3" t="s">
         <v>64</v>
@@ -900,7 +900,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:35" ht="72" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:35" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -953,16 +953,16 @@
         <v>59</v>
       </c>
       <c r="R4">
-        <v>0.29599999999999999</v>
+        <v>0.29399999999999998</v>
       </c>
       <c r="S4">
-        <v>30.8</v>
+        <v>30.9</v>
       </c>
       <c r="T4">
-        <v>15.9</v>
+        <v>13.1</v>
       </c>
       <c r="U4">
-        <v>133.80000000000001</v>
+        <v>103.8</v>
       </c>
       <c r="V4" t="s">
         <v>64</v>
@@ -1007,7 +1007,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:35" ht="72" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:35" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -1060,16 +1060,16 @@
         <v>59</v>
       </c>
       <c r="R5">
-        <v>0.29599999999999999</v>
+        <v>0.29399999999999998</v>
       </c>
       <c r="S5">
-        <v>30.8</v>
+        <v>30.9</v>
       </c>
       <c r="T5">
-        <v>15.9</v>
+        <v>13.1</v>
       </c>
       <c r="U5">
-        <v>133.80000000000001</v>
+        <v>103.8</v>
       </c>
       <c r="V5" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
Stope tracking input_exp_H2-CO2-T32-01500.xlsx file
</commit_message>
<xml_diff>
--- a/input/input_exp_H2-CO2-T32-P1500.xlsx
+++ b/input/input_exp_H2-CO2-T32-P1500.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps2/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="829" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB0A0013-77F2-4C3F-8AF1-733208192591}"/>
+  <xr:revisionPtr revIDLastSave="835" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CF6B8E2-D396-4A24-AD27-3EB19F18CAA9}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="78">
   <si>
     <t>path</t>
   </si>
@@ -264,6 +264,12 @@
   </si>
   <si>
     <t>XP-3340II_20100003_Measurement raw data_20250728114945.csv</t>
+  </si>
+  <si>
+    <t>Angle</t>
+  </si>
+  <si>
+    <t>°</t>
   </si>
 </sst>
 </file>
@@ -607,30 +613,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AJ5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="7.6640625" style="4" customWidth="1"/>
-    <col min="4" max="7" width="7.33203125" customWidth="1"/>
-    <col min="8" max="10" width="7.109375" customWidth="1"/>
-    <col min="11" max="11" width="7.33203125" customWidth="1"/>
-    <col min="12" max="16" width="10.109375" customWidth="1"/>
-    <col min="17" max="21" width="12.88671875" customWidth="1"/>
-    <col min="22" max="25" width="30.33203125" customWidth="1"/>
-    <col min="26" max="26" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="14.5546875" customWidth="1"/>
-    <col min="29" max="29" width="35.33203125" style="1" customWidth="1"/>
-    <col min="30" max="30" width="21.109375" style="1" customWidth="1"/>
-    <col min="31" max="31" width="21.33203125" style="1" customWidth="1"/>
-    <col min="32" max="32" width="26" style="1" customWidth="1"/>
-    <col min="33" max="33" width="18.33203125" style="2" customWidth="1"/>
-    <col min="34" max="34" width="20.33203125" style="2" customWidth="1"/>
-    <col min="35" max="35" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="30.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="7.7109375" style="4" customWidth="1"/>
+    <col min="4" max="8" width="7.28515625" customWidth="1"/>
+    <col min="9" max="11" width="7.140625" customWidth="1"/>
+    <col min="12" max="12" width="7.28515625" customWidth="1"/>
+    <col min="13" max="17" width="10.140625" customWidth="1"/>
+    <col min="18" max="22" width="12.85546875" customWidth="1"/>
+    <col min="23" max="26" width="30.28515625" customWidth="1"/>
+    <col min="27" max="27" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.5703125" customWidth="1"/>
+    <col min="30" max="30" width="35.28515625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="21.140625" style="1" customWidth="1"/>
+    <col min="32" max="32" width="21.28515625" style="1" customWidth="1"/>
+    <col min="33" max="33" width="26" style="1" customWidth="1"/>
+    <col min="34" max="34" width="18.28515625" style="2" customWidth="1"/>
+    <col min="35" max="35" width="20.28515625" style="2" customWidth="1"/>
+    <col min="36" max="36" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -653,91 +659,94 @@
         <v>27</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>12</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>31</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>32</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>34</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>35</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>37</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>39</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>52</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>41</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>42</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>43</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>40</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>45</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>46</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>47</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:35" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:36" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>15</v>
       </c>
@@ -748,32 +757,32 @@
         <v>16</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>48</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K2" s="1"/>
-      <c r="L2" t="s">
-        <v>33</v>
-      </c>
+      <c r="K2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" s="1"/>
       <c r="M2" t="s">
         <v>33</v>
       </c>
-      <c r="O2" t="s">
+      <c r="N2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P2" t="s">
         <v>36</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>38</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>51</v>
-      </c>
-      <c r="S2" t="s">
-        <v>38</v>
       </c>
       <c r="T2" t="s">
         <v>38</v>
@@ -781,19 +790,22 @@
       <c r="U2" t="s">
         <v>38</v>
       </c>
-      <c r="Z2" s="1" t="s">
-        <v>18</v>
+      <c r="V2" t="s">
+        <v>38</v>
       </c>
       <c r="AA2" s="1" t="s">
         <v>18</v>
       </c>
       <c r="AB2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="AC2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="AG2" s="1"/>
       <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
     </row>
-    <row r="3" spans="1:35" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:36" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>53</v>
       </c>
@@ -816,91 +828,94 @@
         <v>1500</v>
       </c>
       <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
         <v>1</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>0</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>100</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>1</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>2</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>6</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>0.193</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>202</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>59.8</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>58</v>
       </c>
-      <c r="R3">
+      <c r="S3">
         <v>0.29399999999999998</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <v>30.9</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>13.1</v>
       </c>
-      <c r="U3">
+      <c r="V3">
         <v>103.8</v>
       </c>
-      <c r="V3" t="s">
+      <c r="W3" t="s">
         <v>59</v>
       </c>
-      <c r="W3">
+      <c r="X3">
         <v>1</v>
       </c>
-      <c r="X3">
+      <c r="Y3">
         <v>2</v>
       </c>
-      <c r="Y3">
+      <c r="Z3">
         <v>3</v>
       </c>
-      <c r="Z3" s="3">
+      <c r="AA3" s="3">
         <v>45860.618796296294</v>
       </c>
-      <c r="AA3" s="3">
+      <c r="AB3" s="3">
         <v>45860.787499999999</v>
       </c>
-      <c r="AB3">
+      <c r="AC3">
         <v>1</v>
       </c>
-      <c r="AC3" s="5" t="s">
+      <c r="AD3" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="AD3" s="5" t="s">
+      <c r="AE3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="AE3" s="5" t="s">
+      <c r="AF3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="AF3" s="5" t="s">
+      <c r="AG3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="AG3" s="6" t="s">
+      <c r="AH3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="AH3" s="6" t="s">
+      <c r="AI3" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="AI3" s="1" t="s">
+      <c r="AJ3" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:35" ht="72" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:36" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>60</v>
       </c>
@@ -923,91 +938,94 @@
         <v>1500</v>
       </c>
       <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
         <v>2</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>0</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>100</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>1</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>2</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>6</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>0.193</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>202</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>59.8</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>58</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <v>0.29399999999999998</v>
       </c>
-      <c r="S4">
+      <c r="T4">
         <v>30.9</v>
       </c>
-      <c r="T4">
+      <c r="U4">
         <v>13.1</v>
       </c>
-      <c r="U4">
+      <c r="V4">
         <v>103.8</v>
       </c>
-      <c r="V4" t="s">
+      <c r="W4" t="s">
         <v>59</v>
       </c>
-      <c r="W4">
+      <c r="X4">
         <v>1</v>
       </c>
-      <c r="X4">
+      <c r="Y4">
         <v>2</v>
       </c>
-      <c r="Y4">
+      <c r="Z4">
         <v>3</v>
       </c>
-      <c r="Z4" s="3">
+      <c r="AA4" s="3">
         <v>45863.485844907409</v>
       </c>
-      <c r="AA4" s="3">
+      <c r="AB4" s="3">
         <v>45863.578865740739</v>
       </c>
-      <c r="AB4">
+      <c r="AC4">
         <v>1</v>
       </c>
-      <c r="AC4" s="5" t="s">
+      <c r="AD4" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="AD4" s="5" t="s">
+      <c r="AE4" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="AE4" s="5" t="s">
+      <c r="AF4" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="AF4" s="5" t="s">
+      <c r="AG4" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="AG4" s="6" t="s">
+      <c r="AH4" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="AH4" s="6" t="s">
+      <c r="AI4" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="AI4" s="1" t="s">
+      <c r="AJ4" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:35" ht="72" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:36" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>68</v>
       </c>
@@ -1030,87 +1048,90 @@
         <v>1500</v>
       </c>
       <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
         <v>5</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>0</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>100</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>1</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <v>2</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>6</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>0.193</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>202</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>59.8</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>58</v>
       </c>
-      <c r="R5">
+      <c r="S5">
         <v>0.29399999999999998</v>
       </c>
-      <c r="S5">
+      <c r="T5">
         <v>30.9</v>
       </c>
-      <c r="T5">
+      <c r="U5">
         <v>13.1</v>
       </c>
-      <c r="U5">
+      <c r="V5">
         <v>103.8</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>59</v>
       </c>
-      <c r="W5">
+      <c r="X5">
         <v>1</v>
       </c>
-      <c r="X5">
+      <c r="Y5">
         <v>2</v>
       </c>
-      <c r="Y5">
+      <c r="Z5">
         <v>3</v>
       </c>
-      <c r="Z5" s="3">
+      <c r="AA5" s="3">
         <v>45866.503113425926</v>
       </c>
-      <c r="AA5" s="3">
+      <c r="AB5" s="3">
         <v>45866.552349537036</v>
       </c>
-      <c r="AB5">
+      <c r="AC5">
         <v>1</v>
       </c>
-      <c r="AC5" s="5" t="s">
+      <c r="AD5" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="AD5" s="1" t="s">
+      <c r="AE5" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="AE5" s="1" t="s">
+      <c r="AF5" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AF5" s="1" t="s">
+      <c r="AG5" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AG5" s="2" t="s">
+      <c r="AH5" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AH5" s="2" t="s">
+      <c r="AI5" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AI5" s="1" t="s">
+      <c r="AJ5" s="1" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>